<commit_message>
Update formula to new 0.15/0.45/0.40 weights with Financial Leverage multiplier
- Replace net_debt_to_financial_score() with net_debt_to_financial_multiplier() (0.8/0.9/1.0/1.1 tiers)
- New formula: (0.15×HQ + 0.45×Rev + 0.40×SC) × Sector × Vol × FinLeverage
- Remove Facility Risk as a standalone component (absorbed into Supply Chain)
- Update benchmark loading for new 8-column Template CGRI.xlsx structure
- Update COMPONENT_KEYS, radar chart dims, stacked bar weights
- Update calculator UI: 3 input tables (no separate Facility Risk table)
- Update methodology page with new formula, weights, and Financial Leverage table
- Add Financial Exposure.xlsx to tracked files; update all Excel files
</commit_message>
<xml_diff>
--- a/data/processed/HQ Country Risk Index.xlsx
+++ b/data/processed/HQ Country Risk Index.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29926"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{282242C4-323A-9043-91A5-5A1116F7DEA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56404DB9-DCD9-4B01-8FD7-12120419FB15}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" firstSheet="1" activeTab="1" xr2:uid="{95916127-3CC4-294F-93BE-B53715E5263E}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="18000" firstSheet="1" activeTab="1" xr2:uid="{95916127-3CC4-294F-93BE-B53715E5263E}"/>
   </bookViews>
   <sheets>
     <sheet name="Geopolitical Risk Index" sheetId="2" r:id="rId1"/>
@@ -580,7 +580,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1861,7 +1861,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="6">
     <dxf>
@@ -2402,13 +2402,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0F843B5-DE71-6C4D-9049-CAF32210F54F}">
   <dimension ref="A1:B148"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="20.100000000000001" thickTop="1">
+    <row r="1" spans="1:2" ht="20" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2416,7 +2416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18">
+    <row r="2" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
@@ -2424,7 +2424,7 @@
         <v>4.37</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18">
+    <row r="3" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>3</v>
       </c>
@@ -2432,7 +2432,7 @@
         <v>5.21</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18">
+    <row r="4" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>4</v>
       </c>
@@ -2440,7 +2440,7 @@
         <v>5.63</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18">
+    <row r="5" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
@@ -2448,7 +2448,7 @@
         <v>4.3600000000000003</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18">
+    <row r="6" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>6</v>
       </c>
@@ -2456,7 +2456,7 @@
         <v>4.79</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="18">
+    <row r="7" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>7</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>3.22</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="18">
+    <row r="8" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>8</v>
       </c>
@@ -2472,7 +2472,7 @@
         <v>3.41</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18">
+    <row r="9" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>9</v>
       </c>
@@ -2480,7 +2480,7 @@
         <v>5.21</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="18">
+    <row r="10" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>10</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>4.26</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="18">
+    <row r="11" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>11</v>
       </c>
@@ -2496,7 +2496,7 @@
         <v>6.29</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="18">
+    <row r="12" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>12</v>
       </c>
@@ -2504,7 +2504,7 @@
         <v>5.45</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="18">
+    <row r="13" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>13</v>
       </c>
@@ -2512,7 +2512,7 @@
         <v>3.33</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="18">
+    <row r="14" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>14</v>
       </c>
@@ -2520,7 +2520,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="18">
+    <row r="15" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>15</v>
       </c>
@@ -2528,7 +2528,7 @@
         <v>5.0199999999999996</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="18">
+    <row r="16" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>16</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>5.41</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="18">
+    <row r="17" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>17</v>
       </c>
@@ -2544,7 +2544,7 @@
         <v>5.34</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="18">
+    <row r="18" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>18</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>4.34</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="18">
+    <row r="19" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>19</v>
       </c>
@@ -2560,7 +2560,7 @@
         <v>5.35</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="18">
+    <row r="20" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>20</v>
       </c>
@@ -2568,7 +2568,7 @@
         <v>4.43</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="18">
+    <row r="21" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>21</v>
       </c>
@@ -2576,7 +2576,7 @@
         <v>6.55</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="18">
+    <row r="22" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>22</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>6.33</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="18">
+    <row r="23" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>23</v>
       </c>
@@ -2592,7 +2592,7 @@
         <v>5.64</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="18">
+    <row r="24" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>24</v>
       </c>
@@ -2600,7 +2600,7 @@
         <v>6.83</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="18">
+    <row r="25" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>25</v>
       </c>
@@ -2608,7 +2608,7 @@
         <v>3.44</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="18">
+    <row r="26" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>26</v>
       </c>
@@ -2616,7 +2616,7 @@
         <v>6.79</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="18">
+    <row r="27" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>27</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>6.84</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="18">
+    <row r="28" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
         <v>28</v>
       </c>
@@ -2632,7 +2632,7 @@
         <v>4.3600000000000003</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="18">
+    <row r="29" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>29</v>
       </c>
@@ -2640,7 +2640,7 @@
         <v>4.26</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="18">
+    <row r="30" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>30</v>
       </c>
@@ -2648,7 +2648,7 @@
         <v>5.72</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="18">
+    <row r="31" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>31</v>
       </c>
@@ -2656,7 +2656,7 @@
         <v>5.65</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="18">
+    <row r="32" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
         <v>32</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>4.2300000000000004</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="18">
+    <row r="33" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>33</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="18">
+    <row r="34" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
         <v>34</v>
       </c>
@@ -2680,7 +2680,7 @@
         <v>4.28</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="18">
+    <row r="35" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
         <v>35</v>
       </c>
@@ -2688,7 +2688,7 @@
         <v>4.67</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="18">
+    <row r="36" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
         <v>36</v>
       </c>
@@ -2696,7 +2696,7 @@
         <v>3.75</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="18">
+    <row r="37" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
         <v>37</v>
       </c>
@@ -2704,7 +2704,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="18">
+    <row r="38" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
         <v>38</v>
       </c>
@@ -2712,7 +2712,7 @@
         <v>5.98</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="18">
+    <row r="39" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
         <v>39</v>
       </c>
@@ -2720,7 +2720,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="18">
+    <row r="40" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
         <v>40</v>
       </c>
@@ -2728,7 +2728,7 @@
         <v>5.71</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="18">
+    <row r="41" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>41</v>
       </c>
@@ -2736,7 +2736,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="18">
+    <row r="42" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
         <v>42</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>4.79</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="18">
+    <row r="43" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
         <v>43</v>
       </c>
@@ -2752,7 +2752,7 @@
         <v>3.57</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="18">
+    <row r="44" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
         <v>44</v>
       </c>
@@ -2760,7 +2760,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="18">
+    <row r="45" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>45</v>
       </c>
@@ -2768,7 +2768,7 @@
         <v>6.93</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="18">
+    <row r="46" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
         <v>46</v>
       </c>
@@ -2776,7 +2776,7 @@
         <v>3.35</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="18">
+    <row r="47" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>47</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>3.65</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="18">
+    <row r="48" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
         <v>48</v>
       </c>
@@ -2792,7 +2792,7 @@
         <v>5.78</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="18">
+    <row r="49" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
         <v>49</v>
       </c>
@@ -2800,7 +2800,7 @@
         <v>5.38</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="18">
+    <row r="50" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
         <v>50</v>
       </c>
@@ -2808,7 +2808,7 @@
         <v>4.93</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="18">
+    <row r="51" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>51</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>3.42</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="18">
+    <row r="52" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
         <v>52</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>4.63</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="18">
+    <row r="53" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
         <v>53</v>
       </c>
@@ -2832,7 +2832,7 @@
         <v>4.34</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="18">
+    <row r="54" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
         <v>54</v>
       </c>
@@ -2840,7 +2840,7 @@
         <v>5.45</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="18">
+    <row r="55" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>55</v>
       </c>
@@ -2848,7 +2848,7 @@
         <v>6.36</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="18">
+    <row r="56" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A56" s="9" t="s">
         <v>56</v>
       </c>
@@ -2856,7 +2856,7 @@
         <v>5.94</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="18">
+    <row r="57" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
         <v>57</v>
       </c>
@@ -2864,7 +2864,7 @@
         <v>4.92</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="18">
+    <row r="58" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A58" s="9" t="s">
         <v>58</v>
       </c>
@@ -2872,7 +2872,7 @@
         <v>6.53</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="18">
+    <row r="59" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
         <v>59</v>
       </c>
@@ -2880,7 +2880,7 @@
         <v>5.77</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="18">
+    <row r="60" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
         <v>60</v>
       </c>
@@ -2888,7 +2888,7 @@
         <v>3.63</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="18">
+    <row r="61" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
         <v>61</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>3.38</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="18">
+    <row r="62" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A62" s="9" t="s">
         <v>62</v>
       </c>
@@ -2904,7 +2904,7 @@
         <v>5.07</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="18">
+    <row r="63" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>63</v>
       </c>
@@ -2912,7 +2912,7 @@
         <v>4.92</v>
       </c>
     </row>
-    <row r="64" spans="1:2" ht="18">
+    <row r="64" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="s">
         <v>64</v>
       </c>
@@ -2920,7 +2920,7 @@
         <v>5.88</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="18">
+    <row r="65" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>65</v>
       </c>
@@ -2928,7 +2928,7 @@
         <v>6.05</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="18">
+    <row r="66" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A66" s="9" t="s">
         <v>66</v>
       </c>
@@ -2936,7 +2936,7 @@
         <v>3.25</v>
       </c>
     </row>
-    <row r="67" spans="1:2" ht="18">
+    <row r="67" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>67</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>4.6100000000000003</v>
       </c>
     </row>
-    <row r="68" spans="1:2" ht="18">
+    <row r="68" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A68" s="9" t="s">
         <v>68</v>
       </c>
@@ -2952,7 +2952,7 @@
         <v>3.84</v>
       </c>
     </row>
-    <row r="69" spans="1:2" ht="18">
+    <row r="69" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>69</v>
       </c>
@@ -2960,7 +2960,7 @@
         <v>4.75</v>
       </c>
     </row>
-    <row r="70" spans="1:2" ht="18">
+    <row r="70" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A70" s="9" t="s">
         <v>70</v>
       </c>
@@ -2968,7 +2968,7 @@
         <v>3.38</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="18">
+    <row r="71" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
         <v>71</v>
       </c>
@@ -2976,7 +2976,7 @@
         <v>5.13</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="18">
+    <row r="72" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A72" s="9" t="s">
         <v>72</v>
       </c>
@@ -2984,7 +2984,7 @@
         <v>4.54</v>
       </c>
     </row>
-    <row r="73" spans="1:2" ht="18">
+    <row r="73" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>73</v>
       </c>
@@ -2992,7 +2992,7 @@
         <v>6.13</v>
       </c>
     </row>
-    <row r="74" spans="1:2" ht="18">
+    <row r="74" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A74" s="9" t="s">
         <v>74</v>
       </c>
@@ -3000,7 +3000,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="75" spans="1:2" ht="18">
+    <row r="75" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
         <v>75</v>
       </c>
@@ -3008,7 +3008,7 @@
         <v>5.37</v>
       </c>
     </row>
-    <row r="76" spans="1:2" ht="18">
+    <row r="76" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A76" s="9" t="s">
         <v>76</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>5.14</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="18">
+    <row r="77" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
         <v>77</v>
       </c>
@@ -3024,7 +3024,7 @@
         <v>3.97</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="18">
+    <row r="78" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A78" s="9" t="s">
         <v>78</v>
       </c>
@@ -3032,7 +3032,7 @@
         <v>6.12</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="18">
+    <row r="79" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
         <v>79</v>
       </c>
@@ -3040,7 +3040,7 @@
         <v>5.49</v>
       </c>
     </row>
-    <row r="80" spans="1:2" ht="18">
+    <row r="80" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A80" s="9" t="s">
         <v>80</v>
       </c>
@@ -3048,7 +3048,7 @@
         <v>5.97</v>
       </c>
     </row>
-    <row r="81" spans="1:2" ht="18">
+    <row r="81" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
         <v>81</v>
       </c>
@@ -3056,7 +3056,7 @@
         <v>5.68</v>
       </c>
     </row>
-    <row r="82" spans="1:2" ht="18">
+    <row r="82" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A82" s="9" t="s">
         <v>82</v>
       </c>
@@ -3064,7 +3064,7 @@
         <v>3.93</v>
       </c>
     </row>
-    <row r="83" spans="1:2" ht="18">
+    <row r="83" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
         <v>83</v>
       </c>
@@ -3072,7 +3072,7 @@
         <v>5.82</v>
       </c>
     </row>
-    <row r="84" spans="1:2" ht="18">
+    <row r="84" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A84" s="9" t="s">
         <v>84</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>5.58</v>
       </c>
     </row>
-    <row r="85" spans="1:2" ht="18">
+    <row r="85" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
         <v>85</v>
       </c>
@@ -3088,7 +3088,7 @@
         <v>4.03</v>
       </c>
     </row>
-    <row r="86" spans="1:2" ht="18">
+    <row r="86" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A86" s="9" t="s">
         <v>86</v>
       </c>
@@ -3096,7 +3096,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="87" spans="1:2" ht="18">
+    <row r="87" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
         <v>87</v>
       </c>
@@ -3104,7 +3104,7 @@
         <v>6.28</v>
       </c>
     </row>
-    <row r="88" spans="1:2" ht="18">
+    <row r="88" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A88" s="9" t="s">
         <v>88</v>
       </c>
@@ -3112,7 +3112,7 @@
         <v>3.47</v>
       </c>
     </row>
-    <row r="89" spans="1:2" ht="18">
+    <row r="89" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
         <v>89</v>
       </c>
@@ -3120,7 +3120,7 @@
         <v>5.42</v>
       </c>
     </row>
-    <row r="90" spans="1:2" ht="18">
+    <row r="90" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A90" s="9" t="s">
         <v>90</v>
       </c>
@@ -3128,7 +3128,7 @@
         <v>5.14</v>
       </c>
     </row>
-    <row r="91" spans="1:2" ht="18">
+    <row r="91" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
         <v>91</v>
       </c>
@@ -3136,7 +3136,7 @@
         <v>4.6500000000000004</v>
       </c>
     </row>
-    <row r="92" spans="1:2" ht="18">
+    <row r="92" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A92" s="9" t="s">
         <v>92</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="93" spans="1:2" ht="18">
+    <row r="93" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
         <v>93</v>
       </c>
@@ -3152,7 +3152,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="94" spans="1:2" ht="18">
+    <row r="94" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A94" s="9" t="s">
         <v>94</v>
       </c>
@@ -3160,7 +3160,7 @@
         <v>4.6399999999999997</v>
       </c>
     </row>
-    <row r="95" spans="1:2" ht="18">
+    <row r="95" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
         <v>95</v>
       </c>
@@ -3168,7 +3168,7 @@
         <v>5.78</v>
       </c>
     </row>
-    <row r="96" spans="1:2" ht="18">
+    <row r="96" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A96" s="9" t="s">
         <v>96</v>
       </c>
@@ -3176,7 +3176,7 @@
         <v>3.59</v>
       </c>
     </row>
-    <row r="97" spans="1:2" ht="18">
+    <row r="97" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
         <v>97</v>
       </c>
@@ -3184,7 +3184,7 @@
         <v>3.32</v>
       </c>
     </row>
-    <row r="98" spans="1:2" ht="18">
+    <row r="98" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A98" s="9" t="s">
         <v>98</v>
       </c>
@@ -3192,7 +3192,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="99" spans="1:2" ht="18">
+    <row r="99" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
         <v>99</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>7.07</v>
       </c>
     </row>
-    <row r="100" spans="1:2" ht="18">
+    <row r="100" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A100" s="9" t="s">
         <v>100</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="101" spans="1:2" ht="18">
+    <row r="101" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A101" s="7" t="s">
         <v>101</v>
       </c>
@@ -3216,7 +3216,7 @@
         <v>4.16</v>
       </c>
     </row>
-    <row r="102" spans="1:2" ht="18">
+    <row r="102" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A102" s="9" t="s">
         <v>102</v>
       </c>
@@ -3224,7 +3224,7 @@
         <v>3.38</v>
       </c>
     </row>
-    <row r="103" spans="1:2" ht="18">
+    <row r="103" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A103" s="7" t="s">
         <v>103</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>4.0199999999999996</v>
       </c>
     </row>
-    <row r="104" spans="1:2" ht="18">
+    <row r="104" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A104" s="9" t="s">
         <v>104</v>
       </c>
@@ -3240,7 +3240,7 @@
         <v>6.65</v>
       </c>
     </row>
-    <row r="105" spans="1:2" ht="18">
+    <row r="105" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A105" s="7" t="s">
         <v>105</v>
       </c>
@@ -3248,7 +3248,7 @@
         <v>4.5599999999999996</v>
       </c>
     </row>
-    <row r="106" spans="1:2" ht="18">
+    <row r="106" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A106" s="9" t="s">
         <v>106</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>5.34</v>
       </c>
     </row>
-    <row r="107" spans="1:2" ht="18">
+    <row r="107" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A107" s="7" t="s">
         <v>107</v>
       </c>
@@ -3264,7 +3264,7 @@
         <v>4.72</v>
       </c>
     </row>
-    <row r="108" spans="1:2" ht="18">
+    <row r="108" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A108" s="9" t="s">
         <v>108</v>
       </c>
@@ -3272,7 +3272,7 @@
         <v>5.28</v>
       </c>
     </row>
-    <row r="109" spans="1:2" ht="18">
+    <row r="109" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A109" s="7" t="s">
         <v>109</v>
       </c>
@@ -3280,7 +3280,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="110" spans="1:2" ht="18">
+    <row r="110" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A110" s="9" t="s">
         <v>110</v>
       </c>
@@ -3288,7 +3288,7 @@
         <v>4.1500000000000004</v>
       </c>
     </row>
-    <row r="111" spans="1:2" ht="18">
+    <row r="111" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A111" s="7" t="s">
         <v>111</v>
       </c>
@@ -3296,7 +3296,7 @@
         <v>3.43</v>
       </c>
     </row>
-    <row r="112" spans="1:2" ht="18">
+    <row r="112" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A112" s="9" t="s">
         <v>112</v>
       </c>
@@ -3304,7 +3304,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="113" spans="1:2" ht="18">
+    <row r="113" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A113" s="7" t="s">
         <v>113</v>
       </c>
@@ -3312,7 +3312,7 @@
         <v>4.05</v>
       </c>
     </row>
-    <row r="114" spans="1:2" ht="18">
+    <row r="114" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A114" s="9" t="s">
         <v>114</v>
       </c>
@@ -3320,7 +3320,7 @@
         <v>5.96</v>
       </c>
     </row>
-    <row r="115" spans="1:2" ht="18">
+    <row r="115" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A115" s="7" t="s">
         <v>115</v>
       </c>
@@ -3328,7 +3328,7 @@
         <v>5.47</v>
       </c>
     </row>
-    <row r="116" spans="1:2" ht="18">
+    <row r="116" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A116" s="9" t="s">
         <v>116</v>
       </c>
@@ -3336,7 +3336,7 @@
         <v>4.42</v>
       </c>
     </row>
-    <row r="117" spans="1:2" ht="18">
+    <row r="117" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A117" s="7" t="s">
         <v>117</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="118" spans="1:2" ht="18">
+    <row r="118" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A118" s="9" t="s">
         <v>118</v>
       </c>
@@ -3352,7 +3352,7 @@
         <v>5.04</v>
       </c>
     </row>
-    <row r="119" spans="1:2" ht="18">
+    <row r="119" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A119" s="7" t="s">
         <v>119</v>
       </c>
@@ -3360,7 +3360,7 @@
         <v>5.64</v>
       </c>
     </row>
-    <row r="120" spans="1:2" ht="18">
+    <row r="120" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A120" s="9" t="s">
         <v>120</v>
       </c>
@@ -3368,7 +3368,7 @@
         <v>3.04</v>
       </c>
     </row>
-    <row r="121" spans="1:2" ht="18">
+    <row r="121" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A121" s="7" t="s">
         <v>121</v>
       </c>
@@ -3376,7 +3376,7 @@
         <v>3.79</v>
       </c>
     </row>
-    <row r="122" spans="1:2" ht="18">
+    <row r="122" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A122" s="9" t="s">
         <v>122</v>
       </c>
@@ -3384,7 +3384,7 @@
         <v>3.48</v>
       </c>
     </row>
-    <row r="123" spans="1:2" ht="18">
+    <row r="123" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A123" s="7" t="s">
         <v>123</v>
       </c>
@@ -3392,7 +3392,7 @@
         <v>5.22</v>
       </c>
     </row>
-    <row r="124" spans="1:2" ht="18">
+    <row r="124" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A124" s="9" t="s">
         <v>124</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>3.57</v>
       </c>
     </row>
-    <row r="125" spans="1:2" ht="18">
+    <row r="125" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A125" s="7" t="s">
         <v>125</v>
       </c>
@@ -3408,7 +3408,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="126" spans="1:2" ht="18">
+    <row r="126" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A126" s="9" t="s">
         <v>126</v>
       </c>
@@ -3416,7 +3416,7 @@
         <v>5.1100000000000003</v>
       </c>
     </row>
-    <row r="127" spans="1:2" ht="18">
+    <row r="127" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A127" s="7" t="s">
         <v>127</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="128" spans="1:2" ht="18">
+    <row r="128" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A128" s="9" t="s">
         <v>128</v>
       </c>
@@ -3432,7 +3432,7 @@
         <v>3.52</v>
       </c>
     </row>
-    <row r="129" spans="1:2" ht="18">
+    <row r="129" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A129" s="7" t="s">
         <v>129</v>
       </c>
@@ -3440,7 +3440,7 @@
         <v>2.78</v>
       </c>
     </row>
-    <row r="130" spans="1:2">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A130" s="118" t="s">
         <v>130</v>
       </c>
@@ -3448,7 +3448,7 @@
         <v>7.33</v>
       </c>
     </row>
-    <row r="131" spans="1:2" ht="18">
+    <row r="131" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A131" s="7" t="s">
         <v>131</v>
       </c>
@@ -3456,7 +3456,7 @@
         <v>5.69</v>
       </c>
     </row>
-    <row r="132" spans="1:2" ht="18">
+    <row r="132" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A132" s="9" t="s">
         <v>132</v>
       </c>
@@ -3464,7 +3464,7 @@
         <v>5.21</v>
       </c>
     </row>
-    <row r="133" spans="1:2" ht="18">
+    <row r="133" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A133" s="7" t="s">
         <v>133</v>
       </c>
@@ -3472,7 +3472,7 @@
         <v>5.15</v>
       </c>
     </row>
-    <row r="134" spans="1:2" ht="18">
+    <row r="134" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A134" s="9" t="s">
         <v>134</v>
       </c>
@@ -3480,7 +3480,7 @@
         <v>5.87</v>
       </c>
     </row>
-    <row r="135" spans="1:2" ht="18">
+    <row r="135" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A135" s="7" t="s">
         <v>135</v>
       </c>
@@ -3488,7 +3488,7 @@
         <v>4.38</v>
       </c>
     </row>
-    <row r="136" spans="1:2" ht="18">
+    <row r="136" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A136" s="9" t="s">
         <v>136</v>
       </c>
@@ -3496,7 +3496,7 @@
         <v>5.13</v>
       </c>
     </row>
-    <row r="137" spans="1:2" ht="18">
+    <row r="137" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A137" s="7" t="s">
         <v>137</v>
       </c>
@@ -3504,7 +3504,7 @@
         <v>5.26</v>
       </c>
     </row>
-    <row r="138" spans="1:2" ht="18">
+    <row r="138" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A138" s="9" t="s">
         <v>138</v>
       </c>
@@ -3512,7 +3512,7 @@
         <v>6.29</v>
       </c>
     </row>
-    <row r="139" spans="1:2" ht="18">
+    <row r="139" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A139" s="7" t="s">
         <v>139</v>
       </c>
@@ -3520,7 +3520,7 @@
         <v>6.35</v>
       </c>
     </row>
-    <row r="140" spans="1:2" ht="18">
+    <row r="140" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A140" s="9" t="s">
         <v>140</v>
       </c>
@@ -3528,7 +3528,7 @@
         <v>3.72</v>
       </c>
     </row>
-    <row r="141" spans="1:2" ht="18">
+    <row r="141" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A141" s="7" t="s">
         <v>141</v>
       </c>
@@ -3536,7 +3536,7 @@
         <v>3.32</v>
       </c>
     </row>
-    <row r="142" spans="1:2" ht="18">
+    <row r="142" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A142" s="9" t="s">
         <v>142</v>
       </c>
@@ -3544,7 +3544,7 @@
         <v>4.1900000000000004</v>
       </c>
     </row>
-    <row r="143" spans="1:2" ht="18">
+    <row r="143" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A143" s="7" t="s">
         <v>143</v>
       </c>
@@ -3552,7 +3552,7 @@
         <v>3.91</v>
       </c>
     </row>
-    <row r="144" spans="1:2" ht="18">
+    <row r="144" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A144" s="9" t="s">
         <v>144</v>
       </c>
@@ -3560,7 +3560,7 @@
         <v>5.77</v>
       </c>
     </row>
-    <row r="145" spans="1:2" ht="18">
+    <row r="145" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A145" s="7" t="s">
         <v>145</v>
       </c>
@@ -3568,7 +3568,7 @@
         <v>4.32</v>
       </c>
     </row>
-    <row r="146" spans="1:2" ht="18">
+    <row r="146" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A146" s="9" t="s">
         <v>146</v>
       </c>
@@ -3576,7 +3576,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="147" spans="1:2" ht="18">
+    <row r="147" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A147" s="7" t="s">
         <v>147</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>4.95</v>
       </c>
     </row>
-    <row r="148" spans="1:2" ht="18">
+    <row r="148" spans="1:2" ht="18" x14ac:dyDescent="0.25">
       <c r="A148" s="9" t="s">
         <v>148</v>
       </c>
@@ -3600,16 +3600,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4742C92E-05CB-2945-90FF-E8780C26B94E}">
   <dimension ref="A1:D26"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="18.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="32.375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="31.875" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="10.875" style="1"/>
+    <col min="2" max="2" width="14.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="32.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="31.83203125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>149</v>
       </c>
@@ -3623,7 +3623,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="135" t="s">
         <v>153</v>
       </c>
@@ -3639,7 +3639,7 @@
         <v>4.1900000000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="135" t="s">
         <v>154</v>
       </c>
@@ -3655,7 +3655,7 @@
         <v>4.1900000000000004</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="135" t="s">
         <v>155</v>
       </c>
@@ -3671,7 +3671,7 @@
         <v>4.1900000000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="135" t="s">
         <v>156</v>
       </c>
@@ -3687,7 +3687,7 @@
         <v>4.1900000000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="135" t="s">
         <v>157</v>
       </c>
@@ -3703,7 +3703,7 @@
         <v>4.1900000000000004</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="135" t="s">
         <v>158</v>
       </c>
@@ -3719,7 +3719,7 @@
         <v>3.57</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="135" t="s">
         <v>159</v>
       </c>
@@ -3735,7 +3735,7 @@
         <v>4.1900000000000004</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="135" t="s">
         <v>160</v>
       </c>
@@ -3751,7 +3751,7 @@
         <v>4.1900000000000004</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="135" t="s">
         <v>161</v>
       </c>
@@ -3767,7 +3767,7 @@
         <v>3.42</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="135" t="s">
         <v>162</v>
       </c>
@@ -3783,7 +3783,7 @@
         <v>3.65</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="135" t="s">
         <v>163</v>
       </c>
@@ -3799,7 +3799,7 @@
         <v>3.65</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="135" t="s">
         <v>164</v>
       </c>
@@ -3815,7 +3815,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="135" t="s">
         <v>165</v>
       </c>
@@ -3831,7 +3831,7 @@
         <v>5.07</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="135" t="s">
         <v>166</v>
       </c>
@@ -3847,7 +3847,7 @@
         <v>4.1900000000000004</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="135" t="s">
         <v>167</v>
       </c>
@@ -3863,7 +3863,7 @@
         <v>3.38</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="135" t="s">
         <v>168</v>
       </c>
@@ -3879,7 +3879,7 @@
         <v>4.26</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="135" t="s">
         <v>169</v>
       </c>
@@ -3895,7 +3895,7 @@
         <v>3.65</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="135" t="s">
         <v>170</v>
       </c>
@@ -3911,7 +3911,7 @@
         <v>3.38</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="135" t="s">
         <v>171</v>
       </c>
@@ -3926,7 +3926,7 @@
         <v>4.26</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="135" t="s">
         <v>173</v>
       </c>
@@ -3942,7 +3942,7 @@
         <v>3.42</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="135" t="s">
         <v>174</v>
       </c>
@@ -3958,7 +3958,7 @@
         <v>4.1900000000000004</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="135" t="s">
         <v>175</v>
       </c>
@@ -3974,7 +3974,7 @@
         <v>3.59</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="135" t="s">
         <v>176</v>
       </c>
@@ -3990,7 +3990,7 @@
         <v>3.65</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="135" t="s">
         <v>177</v>
       </c>
@@ -4006,7 +4006,7 @@
         <v>4.1900000000000004</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="135" t="s">
         <v>178</v>
       </c>
@@ -4043,8 +4043,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100086DC0FFDEFA864DA147FFDEA823F2EE" ma:contentTypeVersion="3" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="efa000e167d9ce5db8cd2eb5b6f87cd4">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c41a64fd-65ba-4a6e-8004-8ade4c8fdb39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f94584ddf2c7798ba84aeef6e679263" ns2:_="">
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100086DC0FFDEFA864DA147FFDEA823F2EE" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="39870545afabb502c4050089500bd5b6">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c41a64fd-65ba-4a6e-8004-8ade4c8fdb39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9bb2a11c505461e40f497f8b9cdcbcf5" ns2:_="">
     <xsd:import namespace="c41a64fd-65ba-4a6e-8004-8ade4c8fdb39"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -4090,8 +4105,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo di contenuto"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titolo"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -4180,29 +4195,44 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0FA7D62-19FC-45A3-82BF-2056044701B9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41CECD9D-ED63-41F4-8222-347F9BB39F2E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="c41a64fd-65ba-4a6e-8004-8ade4c8fdb39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41CECD9D-ED63-41F4-8222-347F9BB39F2E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AD37022-74AD-4B7D-9FDC-188F185CC54B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AD37022-74AD-4B7D-9FDC-188F185CC54B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D4E78C30-5A7A-4066-8785-5A5F06E3C533}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c41a64fd-65ba-4a6e-8004-8ade4c8fdb39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>